<commit_message>
Daily NSE scan: 2026-10-13
</commit_message>
<xml_diff>
--- a/output/2026-10-13/enriched_analysis.xlsx
+++ b/output/2026-10-13/enriched_analysis.xlsx
@@ -929,10 +929,10 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>2.251</v>
+        <v>2.253</v>
       </c>
       <c r="W2" t="n">
-        <v>2799</v>
+        <v>2797</v>
       </c>
       <c r="X2" t="n">
         <v>21.9</v>
@@ -1396,7 +1396,7 @@
         <v>0.044</v>
       </c>
       <c r="W4" t="n">
-        <v>3018</v>
+        <v>3015</v>
       </c>
       <c r="X4" t="n">
         <v>10.4</v>
@@ -1625,13 +1625,13 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>0.533</v>
+        <v>0.529</v>
       </c>
       <c r="W5" t="n">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="X5" t="n">
-        <v>13.6</v>
+        <v>13.7</v>
       </c>
       <c r="Y5" t="n">
         <v>19</v>
@@ -2087,13 +2087,13 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>1.192</v>
+        <v>1.188</v>
       </c>
       <c r="W7" t="n">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="X7" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="Y7" t="n">
         <v>22</v>
@@ -2319,13 +2319,13 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>0.329</v>
+        <v>0.33</v>
       </c>
       <c r="W8" t="n">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="X8" t="n">
-        <v>9.15</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="Y8" t="n">
         <v>7</v>
@@ -2551,13 +2551,13 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>1.167</v>
+        <v>1.173</v>
       </c>
       <c r="W9" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="X9" t="n">
-        <v>7.3</v>
+        <v>7.26</v>
       </c>
       <c r="Y9" t="n">
         <v>17</v>
@@ -2749,7 +2749,7 @@
         <v>-5.9</v>
       </c>
       <c r="L10" t="n">
-        <v>67.16</v>
+        <v>67.31999999999999</v>
       </c>
       <c r="M10" t="n">
         <v>7.21</v>
@@ -2786,7 +2786,7 @@
         <v>0.047</v>
       </c>
       <c r="W10" t="n">
-        <v>15191</v>
+        <v>15201</v>
       </c>
       <c r="X10" t="n">
         <v>38.7</v>
@@ -3015,13 +3015,13 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>2.341</v>
+        <v>2.346</v>
       </c>
       <c r="W11" t="n">
-        <v>2507</v>
+        <v>2502</v>
       </c>
       <c r="X11" t="n">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="Y11" t="n">
         <v>6</v>
@@ -3250,10 +3250,10 @@
         <v>0.05</v>
       </c>
       <c r="W12" t="n">
-        <v>1658</v>
+        <v>1660</v>
       </c>
       <c r="X12" t="n">
-        <v>22.3</v>
+        <v>22.4</v>
       </c>
       <c r="Y12" t="n">
         <v>55</v>
@@ -3482,10 +3482,10 @@
         <v>0.065</v>
       </c>
       <c r="W13" t="n">
-        <v>874</v>
+        <v>870</v>
       </c>
       <c r="X13" t="n">
-        <v>22.1</v>
+        <v>22</v>
       </c>
       <c r="Y13" t="n">
         <v>19</v>
@@ -3709,10 +3709,10 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="W14" t="n">
-        <v>2553</v>
+        <v>2557</v>
       </c>
       <c r="X14" t="n">
         <v>20.9</v>
@@ -4173,13 +4173,13 @@
         </is>
       </c>
       <c r="V16" t="n">
-        <v>0.172</v>
+        <v>0.166</v>
       </c>
       <c r="W16" t="n">
-        <v>646</v>
+        <v>666</v>
       </c>
       <c r="X16" t="n">
-        <v>54</v>
+        <v>55.6</v>
       </c>
       <c r="Y16" t="n">
         <v>3</v>
@@ -4371,7 +4371,7 @@
         <v>-25</v>
       </c>
       <c r="L17" t="n">
-        <v>74.59</v>
+        <v>74.51000000000001</v>
       </c>
       <c r="M17" t="n">
         <v>1.11</v>
@@ -4408,10 +4408,10 @@
         <v>0.068</v>
       </c>
       <c r="W17" t="n">
-        <v>1630</v>
+        <v>1632</v>
       </c>
       <c r="X17" t="n">
-        <v>37.4</v>
+        <v>37.5</v>
       </c>
       <c r="Y17" t="n">
         <v>20</v>
@@ -4637,13 +4637,13 @@
         </is>
       </c>
       <c r="V18" t="n">
-        <v>3.06</v>
+        <v>3.051</v>
       </c>
       <c r="W18" t="n">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="X18" t="n">
-        <v>19.4</v>
+        <v>19.5</v>
       </c>
       <c r="Y18" t="n">
         <v>30</v>
@@ -5096,7 +5096,7 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W20" t="n">
-        <v>54843</v>
+        <v>54825</v>
       </c>
       <c r="X20" t="n">
         <v>46.4</v>
@@ -5328,10 +5328,10 @@
         <v>0.09</v>
       </c>
       <c r="W21" t="n">
-        <v>637</v>
+        <v>632</v>
       </c>
       <c r="X21" t="n">
-        <v>10.4</v>
+        <v>10.3</v>
       </c>
       <c r="Y21" t="n">
         <v>-5</v>
@@ -5523,7 +5523,7 @@
         <v>32.3</v>
       </c>
       <c r="L22" t="n">
-        <v>71.22</v>
+        <v>71.36</v>
       </c>
       <c r="M22" t="n">
         <v>0.86</v>
@@ -5560,7 +5560,7 @@
         <v>0.1</v>
       </c>
       <c r="W22" t="n">
-        <v>860</v>
+        <v>862</v>
       </c>
       <c r="X22" t="n">
         <v>37.5</v>
@@ -5789,7 +5789,7 @@
         <v>186</v>
       </c>
       <c r="X23" t="n">
-        <v>5.45</v>
+        <v>5.43</v>
       </c>
       <c r="Y23" t="n">
         <v>31</v>
@@ -6011,13 +6011,13 @@
         </is>
       </c>
       <c r="V24" t="n">
-        <v>0.303</v>
+        <v>0.318</v>
       </c>
       <c r="W24" t="n">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="X24" t="n">
-        <v>25.3</v>
+        <v>24.1</v>
       </c>
       <c r="Y24" t="n">
         <v>12</v>
@@ -6243,10 +6243,10 @@
         </is>
       </c>
       <c r="V25" t="n">
-        <v>0.41</v>
+        <v>0.409</v>
       </c>
       <c r="W25" t="n">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="X25" t="n">
         <v>48.9</v>
@@ -6478,10 +6478,10 @@
         <v>0.26</v>
       </c>
       <c r="W26" t="n">
-        <v>999</v>
+        <v>1002</v>
       </c>
       <c r="X26" t="n">
-        <v>27.2</v>
+        <v>27.3</v>
       </c>
       <c r="Y26" t="n">
         <v>9</v>
@@ -6710,7 +6710,7 @@
         <v>0.127</v>
       </c>
       <c r="W27" t="n">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="X27" t="n">
         <v>13.9</v>
@@ -6945,7 +6945,7 @@
         <v>380</v>
       </c>
       <c r="X28" t="n">
-        <v>35.2</v>
+        <v>35.3</v>
       </c>
       <c r="Y28" t="n">
         <v>21</v>
@@ -7174,10 +7174,10 @@
         <v>0.042</v>
       </c>
       <c r="W29" t="n">
-        <v>1666</v>
+        <v>1662</v>
       </c>
       <c r="X29" t="n">
-        <v>21.8</v>
+        <v>21.7</v>
       </c>
       <c r="Y29" t="n">
         <v>10</v>
@@ -7870,7 +7870,7 @@
         <v>0.831</v>
       </c>
       <c r="W32" t="n">
-        <v>3804</v>
+        <v>3801</v>
       </c>
       <c r="X32" t="n">
         <v>26.6</v>
@@ -8330,7 +8330,7 @@
         <v>0.237</v>
       </c>
       <c r="W34" t="n">
-        <v>1685</v>
+        <v>1686</v>
       </c>
       <c r="X34" t="n">
         <v>17.8</v>
@@ -8562,7 +8562,7 @@
         <v>0.043</v>
       </c>
       <c r="W35" t="n">
-        <v>3142</v>
+        <v>3140</v>
       </c>
       <c r="X35" t="n">
         <v>18.6</v>
@@ -8791,13 +8791,13 @@
         </is>
       </c>
       <c r="V36" t="n">
-        <v>0.376</v>
+        <v>0.371</v>
       </c>
       <c r="W36" t="n">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="X36" t="n">
-        <v>92.2</v>
+        <v>93.2</v>
       </c>
       <c r="Y36" t="n">
         <v>246</v>
@@ -9252,10 +9252,10 @@
         <v>0</v>
       </c>
       <c r="W38" t="n">
-        <v>5361</v>
+        <v>5355</v>
       </c>
       <c r="X38" t="n">
-        <v>12.6</v>
+        <v>12.5</v>
       </c>
       <c r="Y38" t="n">
         <v>26</v>
@@ -9484,7 +9484,7 @@
         <v>0.011</v>
       </c>
       <c r="W39" t="n">
-        <v>4051</v>
+        <v>4064</v>
       </c>
       <c r="X39" t="inlineStr"/>
       <c r="Y39" t="n">
@@ -9711,13 +9711,13 @@
         </is>
       </c>
       <c r="V40" t="n">
-        <v>0.1</v>
+        <v>0.101</v>
       </c>
       <c r="W40" t="n">
-        <v>496</v>
+        <v>492</v>
       </c>
       <c r="X40" t="n">
-        <v>8.01</v>
+        <v>7.95</v>
       </c>
       <c r="Y40" t="n">
         <v>118</v>
@@ -9905,7 +9905,7 @@
         <v>14.9</v>
       </c>
       <c r="L41" t="n">
-        <v>68.34</v>
+        <v>68.52</v>
       </c>
       <c r="M41" t="n">
         <v>0.2</v>
@@ -10171,13 +10171,13 @@
         </is>
       </c>
       <c r="V42" t="n">
-        <v>0.077</v>
+        <v>0.076</v>
       </c>
       <c r="W42" t="n">
-        <v>437</v>
+        <v>447</v>
       </c>
       <c r="X42" t="n">
-        <v>12.9</v>
+        <v>13.2</v>
       </c>
       <c r="Y42" t="n">
         <v>-8</v>
@@ -10403,13 +10403,13 @@
         </is>
       </c>
       <c r="V43" t="n">
-        <v>0.096</v>
+        <v>0.095</v>
       </c>
       <c r="W43" t="n">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="X43" t="n">
-        <v>28.7</v>
+        <v>28.9</v>
       </c>
       <c r="Y43" t="n">
         <v>24</v>
@@ -10635,10 +10635,10 @@
         </is>
       </c>
       <c r="V44" t="n">
-        <v>0.051</v>
+        <v>0.052</v>
       </c>
       <c r="W44" t="n">
-        <v>959</v>
+        <v>956</v>
       </c>
       <c r="X44" t="inlineStr"/>
       <c r="Y44" t="n">
@@ -10868,10 +10868,10 @@
         <v>0</v>
       </c>
       <c r="W45" t="n">
-        <v>3742</v>
+        <v>3739</v>
       </c>
       <c r="X45" t="n">
-        <v>84.2</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="Y45" t="n">
         <v>42</v>
@@ -11100,7 +11100,7 @@
         <v>0.006</v>
       </c>
       <c r="W46" t="n">
-        <v>4868</v>
+        <v>4863</v>
       </c>
       <c r="X46" t="n">
         <v>12.6</v>
@@ -11328,10 +11328,10 @@
         <v>0</v>
       </c>
       <c r="W47" t="n">
-        <v>103386</v>
+        <v>103284</v>
       </c>
       <c r="X47" t="n">
-        <v>29.8</v>
+        <v>29.7</v>
       </c>
       <c r="Y47" t="n">
         <v>18</v>
@@ -11557,13 +11557,13 @@
         </is>
       </c>
       <c r="V48" t="n">
-        <v>0.239</v>
+        <v>0.235</v>
       </c>
       <c r="W48" t="n">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="X48" t="n">
-        <v>22.4</v>
+        <v>22.8</v>
       </c>
       <c r="Y48" t="n">
         <v>21</v>
@@ -12087,7 +12087,7 @@
         <v>-5.9</v>
       </c>
       <c r="F10" t="n">
-        <v>67.16</v>
+        <v>67.31999999999999</v>
       </c>
       <c r="G10" t="n">
         <v>7.21</v>
@@ -12332,7 +12332,7 @@
         <v>-25</v>
       </c>
       <c r="F17" t="n">
-        <v>74.59</v>
+        <v>74.51000000000001</v>
       </c>
       <c r="G17" t="n">
         <v>1.11</v>
@@ -12507,7 +12507,7 @@
         <v>32.3</v>
       </c>
       <c r="F22" t="n">
-        <v>71.22</v>
+        <v>71.36</v>
       </c>
       <c r="G22" t="n">
         <v>0.86</v>
@@ -13172,7 +13172,7 @@
         <v>14.9</v>
       </c>
       <c r="F41" t="n">
-        <v>68.34</v>
+        <v>68.52</v>
       </c>
       <c r="G41" t="n">
         <v>0.2</v>

</xml_diff>